<commit_message>
#4 Changes Completed and Fresh Deliverables Generated
</commit_message>
<xml_diff>
--- a/Design Files/LLR-05U (Advance Version)/Main Board/BOM/Client BOM LLR-05U (Main-Board).xlsx
+++ b/Design Files/LLR-05U (Advance Version)/Main Board/BOM/Client BOM LLR-05U (Main-Board).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20410"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20411"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\abdullah-liquidlevelrelay\Design Files\LLR-05U (Advance Version)\Main Board\Client BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eSpark Cons Group\Documents\GitHub\Melih-SoundSensor\abdullah-liquidlevelrelay\Design Files\LLR-05U (Advance Version)\Main Board\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96AE7173-7AEC-412D-8E7F-590F6DD138B3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFB5FAED-B925-438E-BA33-A9FBDDA9DA9F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="111">
   <si>
     <t>#</t>
   </si>
@@ -37,6 +37,9 @@
     <t>Diode</t>
   </si>
   <si>
+    <t>Screw Terminal</t>
+  </si>
+  <si>
     <t>Screw terminal</t>
   </si>
   <si>
@@ -52,18 +55,27 @@
     <t>Resistor</t>
   </si>
   <si>
+    <t>NTC Thermistor</t>
+  </si>
+  <si>
     <t>Transformer</t>
   </si>
   <si>
     <t>Optocoupler</t>
   </si>
   <si>
+    <t>Varistors</t>
+  </si>
+  <si>
     <t>Designator</t>
   </si>
   <si>
     <t>C1</t>
   </si>
   <si>
+    <t>C2</t>
+  </si>
+  <si>
     <t>C5</t>
   </si>
   <si>
@@ -103,18 +115,27 @@
     <t>R13, R14</t>
   </si>
   <si>
+    <t>RT1</t>
+  </si>
+  <si>
     <t>T1</t>
   </si>
   <si>
     <t>U1, U2</t>
   </si>
   <si>
+    <t>VR1</t>
+  </si>
+  <si>
     <t>Description</t>
   </si>
   <si>
     <t>330uF 35V ±20% 860mA@100kHz Plugin,D8xL14mm Aluminum Electrolytic Capacitors - Leaded ROHS</t>
   </si>
   <si>
+    <t>5% 400V 100nF PET Plugin,P=7.5mm Film Capacitors ROHS</t>
+  </si>
+  <si>
     <t>47uF 50V ±20% 180mA@100kHz Plugin,D6.3xL12mm Aluminum Electrolytic Capacitors - Leaded ROHS</t>
   </si>
   <si>
@@ -127,10 +148,13 @@
     <t>1A 1.1V@1A 1kV DO-214AC Diodes - General Purpose ROHS</t>
   </si>
   <si>
-    <t>Copper Alloy 1x3P Tin 6.35mm 4 1 3 -40℃~+105℃ 30A 300V Green 10~26 Straight Plugin,P=6.35mm Screw terminal ROHS</t>
-  </si>
-  <si>
-    <t>Copper Alloy 1x2P Tin 6.35mm 4 1 2 -40℃~+105℃ 30A 300V Green 10~26 Straight Plugin,P=6.35mm Screw terminal ROHS</t>
+    <t>1x3P 24A -40℃~+105℃ 250V Green 12~24 Straight 5.08mm 2.5 1 3 Plugin,P=5.08mm Screw terminal ROHS</t>
+  </si>
+  <si>
+    <t>1x2P 24A -40℃~+105℃ 250V Green 12~24 Straight 5.08mm 2.5 1 2 Plugin,P=5.08mm Screw terminal ROHS</t>
+  </si>
+  <si>
+    <t>3A Straight Square Pins 10P 3mm -40℃~+105℃ 3mm 2.54mm 双排 Black 2x5P 2.54mm Plugin,P=2.54mm Pin Headers ROHS</t>
   </si>
   <si>
     <t>12V SPDT (1 Form C) Plugin,15.2x19mm Power Relays ROHS</t>
@@ -151,25 +175,46 @@
     <t>RES SMD 47K OHM 0.1% 1/10W 0603</t>
   </si>
   <si>
+    <t>10Ω 2A 2700K Plugin,P=7.5mm NTC Thermistors ROHS</t>
+  </si>
+  <si>
     <t>Power 2VA 220V / 6Vx2/7.5Vx2/9Vx2/12Vx2/15Vx2/18Vx2/24Vx2 Encapsulated For PCB Mounted Isolation Transformer</t>
   </si>
   <si>
     <t>80V 3.75kV 50mA 300mV@2.4mA,8mA 1 5V 1.25V DC SOP-4-2.54mm Transistor Output Optocoupler ROHS</t>
   </si>
   <si>
+    <t>810V 385V 300V 423V~517V Plugin Varistors ROHS</t>
+  </si>
+  <si>
     <t>Footprint</t>
   </si>
   <si>
     <t>RC035M331LO8*14TH-2A1E</t>
   </si>
   <si>
+    <t>82CL0114</t>
+  </si>
+  <si>
+    <t>Plugin,D6.3xL12mm</t>
+  </si>
+  <si>
+    <t>MBS10S</t>
+  </si>
+  <si>
+    <t>LL-34</t>
+  </si>
+  <si>
     <t>SMA(DO-214AC)</t>
   </si>
   <si>
-    <t>MX635-6.35-03P-GN01-Cu-PS-A</t>
-  </si>
-  <si>
-    <t>MX635-6.35-02P-GN01-Cu-PS-A</t>
+    <t>KF129-5.08-3P</t>
+  </si>
+  <si>
+    <t>KF129-5.08-2P</t>
+  </si>
+  <si>
+    <t>PH-01338</t>
   </si>
   <si>
     <t>HF3FA-012-ZSTF</t>
@@ -187,9 +232,18 @@
     <t>Res-0603</t>
   </si>
   <si>
+    <t>10D-9</t>
+  </si>
+  <si>
     <t>PE2818-I</t>
   </si>
   <si>
+    <t>SOP-4_2.54</t>
+  </si>
+  <si>
+    <t>VDR-05D471K</t>
+  </si>
+  <si>
     <t>Manufacturer Part Number</t>
   </si>
   <si>
@@ -238,7 +292,7 @@
     <t>MSKSEMI</t>
   </si>
   <si>
-    <t>MAX</t>
+    <t>CiXi KaiFeng Electronics</t>
   </si>
   <si>
     <t>Liansheng</t>
@@ -259,15 +313,24 @@
     <t>Yageo</t>
   </si>
   <si>
+    <t>SURGING</t>
+  </si>
+  <si>
     <t>YHDC</t>
   </si>
   <si>
     <t>TOSHIBA</t>
   </si>
   <si>
+    <t>VDR Varistor</t>
+  </si>
+  <si>
     <t>330uF</t>
   </si>
   <si>
+    <t>100nF- 400V</t>
+  </si>
+  <si>
     <t>47uF</t>
   </si>
   <si>
@@ -283,32 +346,20 @@
     <t>47K</t>
   </si>
   <si>
+    <t>PE2818-I 2VA 220V 12Vx2</t>
+  </si>
+  <si>
     <t>Quantity</t>
   </si>
   <si>
-    <t>Remarks</t>
-  </si>
-  <si>
     <t>Value</t>
-  </si>
-  <si>
-    <t>Custom</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>Straight Square Pins 10P, 40mm total length of the pins, 2.54mm pitch, Black 2x5P 2.54mm Plugin,P=2.54mm Pin Headers</t>
-  </si>
-  <si>
-    <t>This pin header is unavailable on LCSC. To source it, we have to consider the following link: https://www.aliexpress.us/item/3256804657327800.html?gatewayAdapt=4itemAdapt</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -351,14 +402,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -472,11 +515,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -516,10 +558,8 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -805,7 +845,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
@@ -815,12 +855,11 @@
     <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="29.7109375" customWidth="1"/>
+    <col min="9" max="9" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -831,9 +870,8 @@
       <c r="H1" s="2"/>
       <c r="I1" s="14"/>
       <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-    </row>
-    <row r="2" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -842,31 +880,28 @@
         <v>1</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>89</v>
+        <v>110</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="11">
         <f>ROW(B3) - ROW($B$2)</f>
@@ -876,125 +911,121 @@
         <v>2</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>90</v>
+        <v>56</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>81</v>
+        <v>101</v>
       </c>
       <c r="J3" s="7">
         <v>1</v>
       </c>
-      <c r="K3" s="7"/>
-    </row>
-    <row r="4" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
-        <f t="shared" ref="B4:B18" si="0">ROW(B4) - ROW($B$2)</f>
+        <f t="shared" ref="B4:B20" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="12" t="s">
         <v>2</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>90</v>
+        <v>57</v>
       </c>
       <c r="G4" s="10" t="s">
         <v>57</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>82</v>
+        <v>102</v>
       </c>
       <c r="J4" s="9">
         <v>1</v>
       </c>
-      <c r="K4" s="9"/>
-    </row>
-    <row r="5" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:10" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="11">
         <f>ROW(B5) - ROW($B$2)</f>
         <v>3</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>90</v>
+        <v>58</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>58</v>
+        <v>103</v>
       </c>
       <c r="J5" s="7">
-        <v>2</v>
-      </c>
-      <c r="K5" s="7"/>
-    </row>
-    <row r="6" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="11">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>90</v>
+        <v>59</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="J6" s="9">
-        <v>1</v>
-      </c>
-      <c r="K6" s="9"/>
-    </row>
-    <row r="7" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="11">
         <f>ROW(B7) - ROW($B$2)</f>
@@ -1004,61 +1035,59 @@
         <v>4</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="J7" s="7">
-        <v>3</v>
-      </c>
-      <c r="K7" s="7"/>
-    </row>
-    <row r="8" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="11">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>90</v>
+        <v>61</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>48</v>
+        <v>78</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="J8" s="9">
-        <v>2</v>
-      </c>
-      <c r="K8" s="9"/>
-    </row>
-    <row r="9" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="11">
         <f>ROW(B9) - ROW($B$2)</f>
@@ -1068,29 +1097,28 @@
         <v>5</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="F9" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="H9" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="G9" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="I9" s="10" t="s">
-        <v>91</v>
+      <c r="I9" s="8" t="s">
+        <v>62</v>
       </c>
       <c r="J9" s="7">
-        <v>1</v>
-      </c>
-      <c r="K9" s="7"/>
-    </row>
-    <row r="10" spans="1:13" ht="72.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="11">
         <f t="shared" si="0"/>
@@ -1100,32 +1128,28 @@
         <v>6</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>92</v>
+        <v>43</v>
       </c>
       <c r="F10" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="H10" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="G10" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="H10" s="9" t="s">
-        <v>73</v>
-      </c>
       <c r="I10" s="10" t="s">
-        <v>91</v>
+        <v>63</v>
       </c>
       <c r="J10" s="9">
         <v>1</v>
       </c>
-      <c r="K10" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="M10" s="15"/>
-    </row>
-    <row r="11" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:10" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="11">
         <f>ROW(B11) - ROW($B$2)</f>
@@ -1135,29 +1159,28 @@
         <v>7</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>90</v>
+        <v>64</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="I11" s="10" t="s">
         <v>91</v>
+      </c>
+      <c r="I11" s="8" t="s">
+        <v>64</v>
       </c>
       <c r="J11" s="7">
         <v>1</v>
       </c>
-      <c r="K11" s="7"/>
-    </row>
-    <row r="12" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="11">
         <f t="shared" si="0"/>
@@ -1167,29 +1190,28 @@
         <v>8</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>61</v>
+        <v>65</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>65</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>91</v>
+        <v>65</v>
       </c>
       <c r="J12" s="9">
-        <v>2</v>
-      </c>
-      <c r="K12" s="9"/>
-    </row>
-    <row r="13" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="11">
         <f>ROW(B13) - ROW($B$2)</f>
@@ -1199,125 +1221,121 @@
         <v>9</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>52</v>
+        <v>66</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>76</v>
+        <v>93</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="J13" s="7">
-        <v>1</v>
-      </c>
-      <c r="K13" s="7"/>
-    </row>
-    <row r="14" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="11">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>63</v>
+        <v>80</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>77</v>
+        <v>94</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>84</v>
+        <v>104</v>
       </c>
       <c r="J14" s="9">
-        <v>2</v>
-      </c>
-      <c r="K14" s="9"/>
-    </row>
-    <row r="15" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="11">
         <f>ROW(B15) - ROW($B$2)</f>
         <v>13</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>64</v>
+        <v>81</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>78</v>
+        <v>95</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>85</v>
+        <v>105</v>
       </c>
       <c r="J15" s="7">
         <v>2</v>
       </c>
-      <c r="K15" s="7"/>
-    </row>
-    <row r="16" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="11">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>65</v>
+        <v>82</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>86</v>
+        <v>106</v>
       </c>
       <c r="J16" s="9">
         <v>2</v>
       </c>
-      <c r="K16" s="9"/>
-    </row>
-    <row r="17" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="11">
         <f>ROW(B17) - ROW($B$2)</f>
@@ -1327,29 +1345,28 @@
         <v>10</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>90</v>
+        <v>69</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>55</v>
+        <v>83</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>91</v>
+        <v>107</v>
       </c>
       <c r="J17" s="7">
-        <v>1</v>
-      </c>
-      <c r="K17" s="7"/>
-    </row>
-    <row r="18" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="11">
         <f t="shared" si="0"/>
@@ -1359,31 +1376,123 @@
         <v>11</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="I18" s="8" t="s">
-        <v>91</v>
+        <v>97</v>
+      </c>
+      <c r="I18" s="10" t="s">
+        <v>104</v>
       </c>
       <c r="J18" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="1"/>
+      <c r="B19" s="11">
+        <f>ROW(B19) - ROW($B$2)</f>
+        <v>17</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="I19" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="J19" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="1"/>
+      <c r="B20" s="11">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="G20" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="H20" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="I20" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="J20" s="9">
         <v>2</v>
       </c>
-      <c r="K18" s="9"/>
+    </row>
+    <row r="21" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="1"/>
+      <c r="B21" s="11">
+        <f>ROW(B21) - ROW($B$2)</f>
+        <v>19</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="G21" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="I21" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="J21" s="7">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I1:J1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>